<commit_message>
unhidden sheet changed to hidden
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-ja_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-ja_my-app.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{554C91CB-6C7B-1F46-871F-FC33190DB484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E6D80B-00B6-3248-8FD2-39F50E0E6587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="6860" windowWidth="28800" windowHeight="10300" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2320" windowWidth="28800" windowHeight="14820" tabRatio="853" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="dataTypeプルダウン項目" sheetId="1" r:id="rId1"/>
+    <sheet name="dataTypeプルダウン項目" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="dataType・データパターン一覧" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="FK種類" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="fmt変更履歴" sheetId="4" r:id="rId4"/>

</xml_diff>